<commit_message>
Update MLB pipeline outputs for 2026-10-30
Re-ran pipeline scripts: verify-facts (25 claims), compile-content-data,
generate-review-dashboard, PostPlanner exports (17 posts / 12 TOBI).
Appended Oct 30 stories to story-history.md. WordPress publish and
dashboard push blocked by proxy (known restriction).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wnm36dD6qFnLrmrKwUgcyH
</commit_message>
<xml_diff>
--- a/MLB/postplanner-imports/bb-postplanner-2026-10-30.xlsx
+++ b/MLB/postplanner-imports/bb-postplanner-2026-10-30.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10/30/2026  10:53</t>
+          <t>10/30/2026  10:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -492,7 +492,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10/30/2026  11:32</t>
+          <t>10/30/2026  11:34</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,7 +508,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10/30/2026  12:11</t>
+          <t>10/30/2026  12:13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -520,7 +520,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10/30/2026  12:50</t>
+          <t>10/30/2026  12:52</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -534,7 +534,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10/30/2026  13:29</t>
+          <t>10/30/2026  13:31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10/30/2026  14:08</t>
+          <t>10/30/2026  14:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -562,7 +562,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10/30/2026  14:47</t>
+          <t>10/30/2026  14:49</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -577,7 +577,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10/30/2026  15:26</t>
+          <t>10/30/2026  15:28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -591,7 +591,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10/30/2026  16:05</t>
+          <t>10/30/2026  16:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -607,7 +607,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10/30/2026  16:44</t>
+          <t>10/30/2026  16:46</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10/30/2026  17:23</t>
+          <t>10/30/2026  17:25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10/30/2026  18:02</t>
+          <t>10/30/2026  18:04</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10/30/2026  18:41</t>
+          <t>10/30/2026  18:43</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -663,7 +663,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10/30/2026  19:20</t>
+          <t>10/30/2026  19:22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -675,7 +675,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10/30/2026  19:59</t>
+          <t>10/30/2026  20:01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -689,7 +689,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10/30/2026  20:38</t>
+          <t>10/30/2026  20:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -705,7 +705,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10/30/2026  21:17</t>
+          <t>10/30/2026  21:19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>